<commit_message>
New system for vsr points
</commit_message>
<xml_diff>
--- a/file/players_updated.xlsx
+++ b/file/players_updated.xlsx
@@ -38565,10 +38565,10 @@
         <v>anchor</v>
       </c>
       <c r="D588">
-        <v>240</v>
+        <v>2382.8571428571427</v>
       </c>
       <c r="E588">
-        <v>240</v>
+        <v>2382.8571428571427</v>
       </c>
       <c r="F588">
         <v>5</v>
@@ -38583,7 +38583,7 @@
         <v>0</v>
       </c>
       <c r="J588">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K588">
         <v>1</v>
@@ -39735,10 +39735,10 @@
         <v>rifler</v>
       </c>
       <c r="D606">
-        <v>120</v>
+        <v>2262.8571428571427</v>
       </c>
       <c r="E606">
-        <v>120</v>
+        <v>2262.8571428571427</v>
       </c>
       <c r="F606">
         <v>5</v>
@@ -39753,7 +39753,7 @@
         <v>0</v>
       </c>
       <c r="J606">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K606">
         <v>0</v>
@@ -53125,10 +53125,10 @@
         <v>rifler</v>
       </c>
       <c r="D812">
-        <v>160</v>
+        <v>2302.8571428571427</v>
       </c>
       <c r="E812">
-        <v>160</v>
+        <v>2302.8571428571427</v>
       </c>
       <c r="F812">
         <v>5</v>
@@ -53143,7 +53143,7 @@
         <v>0</v>
       </c>
       <c r="J812">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K812">
         <v>0</v>
@@ -53190,10 +53190,10 @@
         <v>awper</v>
       </c>
       <c r="D813">
-        <v>160</v>
+        <v>3731.428571428571</v>
       </c>
       <c r="E813">
-        <v>160</v>
+        <v>3731.428571428571</v>
       </c>
       <c r="F813">
         <v>5</v>
@@ -53205,7 +53205,7 @@
         <v>0</v>
       </c>
       <c r="I813">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J813">
         <v>0</v>
@@ -53255,10 +53255,10 @@
         <v>entry fragger</v>
       </c>
       <c r="D814">
-        <v>160</v>
+        <v>5160</v>
       </c>
       <c r="E814">
-        <v>160</v>
+        <v>5160</v>
       </c>
       <c r="F814">
         <v>5</v>
@@ -53267,7 +53267,7 @@
         <v>kONO</v>
       </c>
       <c r="H814">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I814">
         <v>0</v>

</xml_diff>